<commit_message>
Implemented initial version of attractive and repulsive pheromones
</commit_message>
<xml_diff>
--- a/experiments/all_experiments.xlsx
+++ b/experiments/all_experiments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eashw\Desktop\post_graduation_plan\Collaborations\Swarm_collaboration_via_stigmergy\experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB64B812-CC51-4810-BFA6-7D6B9D51BCA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E5A319-7130-47D9-98B5-44E0D4F0D3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -333,18 +333,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -359,6 +347,18 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1974,32 +1974,32 @@
       <c r="F9" s="1"/>
     </row>
     <row r="11" spans="2:20" ht="18.3" x14ac:dyDescent="0.7">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16" t="s">
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16" t="s">
+      <c r="G11" s="21"/>
+      <c r="H11" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="17" t="s">
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="21"/>
+      <c r="O11" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
-      <c r="S11" s="19"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="23"/>
+      <c r="R11" s="23"/>
+      <c r="S11" s="24"/>
     </row>
     <row r="12" spans="2:20" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="3" t="s">
@@ -2041,22 +2041,22 @@
       <c r="N12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="O12" s="22" t="s">
+      <c r="O12" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P12" s="22" t="s">
+      <c r="P12" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q12" s="22" t="s">
+      <c r="Q12" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R12" s="22" t="s">
+      <c r="R12" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S12" s="22" t="s">
+      <c r="S12" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T12" s="23"/>
+      <c r="T12" s="19"/>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" s="4">
@@ -2074,7 +2074,7 @@
       <c r="F13" s="12">
         <v>1</v>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="16">
         <v>104</v>
       </c>
       <c r="H13" s="4">
@@ -2098,22 +2098,22 @@
       <c r="N13" s="14">
         <v>509.68009574634158</v>
       </c>
-      <c r="O13" s="23">
-        <v>5</v>
-      </c>
-      <c r="P13" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q13" s="23">
-        <v>5</v>
-      </c>
-      <c r="R13" s="23">
+      <c r="O13" s="19">
+        <v>5</v>
+      </c>
+      <c r="P13" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q13" s="19">
+        <v>5</v>
+      </c>
+      <c r="R13" s="19">
         <v>1131.5999999999999</v>
       </c>
-      <c r="S13" s="24">
+      <c r="S13" s="20">
         <v>435.12906131399677</v>
       </c>
-      <c r="T13" s="23"/>
+      <c r="T13" s="19"/>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" s="4">
@@ -2131,7 +2131,7 @@
       <c r="F14" s="12">
         <v>1</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="16">
         <v>317</v>
       </c>
       <c r="H14" s="4">
@@ -2155,22 +2155,22 @@
       <c r="N14" s="14">
         <v>693.3639015697313</v>
       </c>
-      <c r="O14" s="23">
-        <v>5</v>
-      </c>
-      <c r="P14" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q14" s="23">
-        <v>5</v>
-      </c>
-      <c r="R14" s="23">
+      <c r="O14" s="19">
+        <v>5</v>
+      </c>
+      <c r="P14" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q14" s="19">
+        <v>5</v>
+      </c>
+      <c r="R14" s="19">
         <v>2725.2</v>
       </c>
-      <c r="S14" s="24">
+      <c r="S14" s="20">
         <v>597.21034820237332</v>
       </c>
-      <c r="T14" s="23"/>
+      <c r="T14" s="19"/>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="4">
@@ -2188,7 +2188,7 @@
       <c r="F15" s="12">
         <v>1</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="16">
         <v>567</v>
       </c>
       <c r="H15" s="4">
@@ -2212,22 +2212,22 @@
       <c r="N15" s="14">
         <v>2074.7313802032299</v>
       </c>
-      <c r="O15" s="23">
-        <v>5</v>
-      </c>
-      <c r="P15" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q15" s="23">
-        <v>5</v>
-      </c>
-      <c r="R15" s="23">
+      <c r="O15" s="19">
+        <v>5</v>
+      </c>
+      <c r="P15" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="19">
+        <v>5</v>
+      </c>
+      <c r="R15" s="19">
         <v>6355.6</v>
       </c>
-      <c r="S15" s="24">
+      <c r="S15" s="20">
         <v>1176.350202958286</v>
       </c>
-      <c r="T15" s="23"/>
+      <c r="T15" s="19"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.55000000000000004">
       <c r="B16" s="7">
@@ -2245,7 +2245,7 @@
       <c r="F16" s="13">
         <v>1</v>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="17">
         <v>704</v>
       </c>
       <c r="H16" s="7">
@@ -2269,708 +2269,708 @@
       <c r="N16" s="15">
         <v>1180.335206625643</v>
       </c>
-      <c r="O16" s="23">
-        <v>5</v>
-      </c>
-      <c r="P16" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q16" s="23">
-        <v>5</v>
-      </c>
-      <c r="R16" s="23">
+      <c r="O16" s="19">
+        <v>5</v>
+      </c>
+      <c r="P16" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q16" s="19">
+        <v>5</v>
+      </c>
+      <c r="R16" s="19">
         <v>9869.4</v>
       </c>
-      <c r="S16" s="24">
+      <c r="S16" s="20">
         <v>1870.953981261966</v>
       </c>
-      <c r="T16" s="23"/>
+      <c r="T16" s="19"/>
     </row>
     <row r="17" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O17" s="23"/>
-      <c r="P17" s="23"/>
-      <c r="Q17" s="23"/>
-      <c r="R17" s="23"/>
-      <c r="S17" s="23"/>
-      <c r="T17" s="23"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="19"/>
+      <c r="S17" s="19"/>
+      <c r="T17" s="19"/>
     </row>
     <row r="18" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O18" s="22" t="s">
+      <c r="O18" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P18" s="22" t="s">
+      <c r="P18" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q18" s="22" t="s">
+      <c r="Q18" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R18" s="22" t="s">
+      <c r="R18" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S18" s="22" t="s">
+      <c r="S18" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T18" s="23"/>
+      <c r="T18" s="19"/>
     </row>
     <row r="19" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O19" s="23">
-        <v>5</v>
-      </c>
-      <c r="P19" s="23">
+      <c r="O19" s="19">
+        <v>5</v>
+      </c>
+      <c r="P19" s="19">
         <v>10</v>
       </c>
-      <c r="Q19" s="23">
-        <v>5</v>
-      </c>
-      <c r="R19" s="23">
+      <c r="Q19" s="19">
+        <v>5</v>
+      </c>
+      <c r="R19" s="19">
         <v>1447.8</v>
       </c>
-      <c r="S19" s="24">
+      <c r="S19" s="20">
         <v>613.87026316641209</v>
       </c>
-      <c r="T19" s="23"/>
+      <c r="T19" s="19"/>
     </row>
     <row r="20" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O20" s="23">
-        <v>5</v>
-      </c>
-      <c r="P20" s="23">
+      <c r="O20" s="19">
+        <v>5</v>
+      </c>
+      <c r="P20" s="19">
         <v>10</v>
       </c>
-      <c r="Q20" s="23">
-        <v>5</v>
-      </c>
-      <c r="R20" s="23">
+      <c r="Q20" s="19">
+        <v>5</v>
+      </c>
+      <c r="R20" s="19">
         <v>3209.4</v>
       </c>
-      <c r="S20" s="24">
+      <c r="S20" s="20">
         <v>451.98816356183482</v>
       </c>
-      <c r="T20" s="23"/>
+      <c r="T20" s="19"/>
     </row>
     <row r="21" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O21" s="23">
-        <v>5</v>
-      </c>
-      <c r="P21" s="23">
+      <c r="O21" s="19">
+        <v>5</v>
+      </c>
+      <c r="P21" s="19">
         <v>10</v>
       </c>
-      <c r="Q21" s="23">
-        <v>5</v>
-      </c>
-      <c r="R21" s="23">
+      <c r="Q21" s="19">
+        <v>5</v>
+      </c>
+      <c r="R21" s="19">
         <v>9413</v>
       </c>
-      <c r="S21" s="24">
+      <c r="S21" s="20">
         <v>6244.8564835390735</v>
       </c>
-      <c r="T21" s="23"/>
+      <c r="T21" s="19"/>
     </row>
     <row r="22" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O22" s="23">
-        <v>5</v>
-      </c>
-      <c r="P22" s="23">
+      <c r="O22" s="19">
+        <v>5</v>
+      </c>
+      <c r="P22" s="19">
         <v>10</v>
       </c>
-      <c r="Q22" s="23">
-        <v>5</v>
-      </c>
-      <c r="R22" s="23">
+      <c r="Q22" s="19">
+        <v>5</v>
+      </c>
+      <c r="R22" s="19">
         <v>10243.799999999999</v>
       </c>
-      <c r="S22" s="24">
+      <c r="S22" s="20">
         <v>3801.8639112940382</v>
       </c>
-      <c r="T22" s="23"/>
+      <c r="T22" s="19"/>
     </row>
     <row r="23" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O23" s="23"/>
-      <c r="P23" s="23"/>
-      <c r="Q23" s="23"/>
-      <c r="R23" s="23"/>
-      <c r="S23" s="23"/>
-      <c r="T23" s="23"/>
+      <c r="O23" s="19"/>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="19"/>
     </row>
     <row r="24" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O24" s="22" t="s">
+      <c r="O24" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P24" s="22" t="s">
+      <c r="P24" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q24" s="22" t="s">
+      <c r="Q24" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R24" s="22" t="s">
+      <c r="R24" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S24" s="22" t="s">
+      <c r="S24" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T24" s="23"/>
+      <c r="T24" s="19"/>
     </row>
     <row r="25" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O25" s="23">
-        <v>5</v>
-      </c>
-      <c r="P25" s="23">
+      <c r="O25" s="19">
+        <v>5</v>
+      </c>
+      <c r="P25" s="19">
         <v>15</v>
       </c>
-      <c r="Q25" s="23">
-        <v>5</v>
-      </c>
-      <c r="R25" s="23">
+      <c r="Q25" s="19">
+        <v>5</v>
+      </c>
+      <c r="R25" s="19">
         <v>1198.8</v>
       </c>
-      <c r="S25" s="24">
+      <c r="S25" s="20">
         <v>390.56523142747869</v>
       </c>
-      <c r="T25" s="23"/>
+      <c r="T25" s="19"/>
     </row>
     <row r="26" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O26" s="23">
-        <v>5</v>
-      </c>
-      <c r="P26" s="23">
+      <c r="O26" s="19">
+        <v>5</v>
+      </c>
+      <c r="P26" s="19">
         <v>15</v>
       </c>
-      <c r="Q26" s="23">
-        <v>5</v>
-      </c>
-      <c r="R26" s="23">
+      <c r="Q26" s="19">
+        <v>5</v>
+      </c>
+      <c r="R26" s="19">
         <v>4550.6000000000004</v>
       </c>
-      <c r="S26" s="24">
+      <c r="S26" s="20">
         <v>2428.0715187160358</v>
       </c>
-      <c r="T26" s="23"/>
+      <c r="T26" s="19"/>
     </row>
     <row r="27" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O27" s="23">
-        <v>5</v>
-      </c>
-      <c r="P27" s="23">
+      <c r="O27" s="19">
+        <v>5</v>
+      </c>
+      <c r="P27" s="19">
         <v>15</v>
       </c>
-      <c r="Q27" s="23">
-        <v>5</v>
-      </c>
-      <c r="R27" s="23">
+      <c r="Q27" s="19">
+        <v>5</v>
+      </c>
+      <c r="R27" s="19">
         <v>5037.3999999999996</v>
       </c>
-      <c r="S27" s="24">
+      <c r="S27" s="20">
         <v>1823.3623611339569</v>
       </c>
-      <c r="T27" s="23"/>
+      <c r="T27" s="19"/>
     </row>
     <row r="28" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O28" s="23">
-        <v>5</v>
-      </c>
-      <c r="P28" s="23">
+      <c r="O28" s="19">
+        <v>5</v>
+      </c>
+      <c r="P28" s="19">
         <v>15</v>
       </c>
-      <c r="Q28" s="23">
-        <v>5</v>
-      </c>
-      <c r="R28" s="23">
+      <c r="Q28" s="19">
+        <v>5</v>
+      </c>
+      <c r="R28" s="19">
         <v>9604.7999999999993</v>
       </c>
-      <c r="S28" s="24">
+      <c r="S28" s="20">
         <v>2373.114767557608</v>
       </c>
-      <c r="T28" s="23"/>
+      <c r="T28" s="19"/>
     </row>
     <row r="29" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O29" s="23"/>
-      <c r="P29" s="23"/>
-      <c r="Q29" s="23"/>
-      <c r="R29" s="23"/>
-      <c r="S29" s="23"/>
-      <c r="T29" s="23"/>
+      <c r="O29" s="19"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="19"/>
+      <c r="R29" s="19"/>
+      <c r="S29" s="19"/>
+      <c r="T29" s="19"/>
     </row>
     <row r="30" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O30" s="22" t="s">
+      <c r="O30" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P30" s="22" t="s">
+      <c r="P30" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q30" s="22" t="s">
+      <c r="Q30" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R30" s="22" t="s">
+      <c r="R30" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S30" s="22" t="s">
+      <c r="S30" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T30" s="23"/>
+      <c r="T30" s="19"/>
     </row>
     <row r="31" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O31" s="23">
-        <v>5</v>
-      </c>
-      <c r="P31" s="23">
+      <c r="O31" s="19">
+        <v>5</v>
+      </c>
+      <c r="P31" s="19">
         <v>20</v>
       </c>
-      <c r="Q31" s="23">
-        <v>5</v>
-      </c>
-      <c r="R31" s="23">
+      <c r="Q31" s="19">
+        <v>5</v>
+      </c>
+      <c r="R31" s="19">
         <v>1702.6</v>
       </c>
-      <c r="S31" s="24">
+      <c r="S31" s="20">
         <v>495.82335564190601</v>
       </c>
-      <c r="T31" s="23"/>
+      <c r="T31" s="19"/>
     </row>
     <row r="32" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O32" s="23">
-        <v>5</v>
-      </c>
-      <c r="P32" s="23">
+      <c r="O32" s="19">
+        <v>5</v>
+      </c>
+      <c r="P32" s="19">
         <v>20</v>
       </c>
-      <c r="Q32" s="23">
-        <v>5</v>
-      </c>
-      <c r="R32" s="23">
+      <c r="Q32" s="19">
+        <v>5</v>
+      </c>
+      <c r="R32" s="19">
         <v>4783</v>
       </c>
-      <c r="S32" s="24">
+      <c r="S32" s="20">
         <v>2185.6666031213449</v>
       </c>
-      <c r="T32" s="23"/>
+      <c r="T32" s="19"/>
     </row>
     <row r="33" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O33" s="23">
-        <v>5</v>
-      </c>
-      <c r="P33" s="23">
+      <c r="O33" s="19">
+        <v>5</v>
+      </c>
+      <c r="P33" s="19">
         <v>20</v>
       </c>
-      <c r="Q33" s="23">
-        <v>5</v>
-      </c>
-      <c r="R33" s="23">
+      <c r="Q33" s="19">
+        <v>5</v>
+      </c>
+      <c r="R33" s="19">
         <v>8204</v>
       </c>
-      <c r="S33" s="24">
+      <c r="S33" s="20">
         <v>2690.5235549981721</v>
       </c>
-      <c r="T33" s="23"/>
+      <c r="T33" s="19"/>
     </row>
     <row r="34" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O34" s="23">
-        <v>5</v>
-      </c>
-      <c r="P34" s="23">
+      <c r="O34" s="19">
+        <v>5</v>
+      </c>
+      <c r="P34" s="19">
         <v>20</v>
       </c>
-      <c r="Q34" s="23">
-        <v>5</v>
-      </c>
-      <c r="R34" s="23">
+      <c r="Q34" s="19">
+        <v>5</v>
+      </c>
+      <c r="R34" s="19">
         <v>8364.2000000000007</v>
       </c>
-      <c r="S34" s="24">
+      <c r="S34" s="20">
         <v>2087.489329314044</v>
       </c>
-      <c r="T34" s="23"/>
+      <c r="T34" s="19"/>
     </row>
     <row r="35" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O35" s="23"/>
-      <c r="P35" s="23"/>
-      <c r="Q35" s="23"/>
-      <c r="R35" s="23"/>
-      <c r="S35" s="23"/>
-      <c r="T35" s="23"/>
+      <c r="O35" s="19"/>
+      <c r="P35" s="19"/>
+      <c r="Q35" s="19"/>
+      <c r="R35" s="19"/>
+      <c r="S35" s="19"/>
+      <c r="T35" s="19"/>
     </row>
     <row r="36" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O36" s="22" t="s">
+      <c r="O36" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P36" s="22" t="s">
+      <c r="P36" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q36" s="22" t="s">
+      <c r="Q36" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R36" s="22" t="s">
+      <c r="R36" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S36" s="22" t="s">
+      <c r="S36" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T36" s="23"/>
+      <c r="T36" s="19"/>
     </row>
     <row r="37" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O37" s="23">
+      <c r="O37" s="19">
         <v>20</v>
       </c>
-      <c r="P37" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q37" s="23">
-        <v>5</v>
-      </c>
-      <c r="R37" s="23">
+      <c r="P37" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q37" s="19">
+        <v>5</v>
+      </c>
+      <c r="R37" s="19">
         <v>1305.4000000000001</v>
       </c>
-      <c r="S37" s="24">
+      <c r="S37" s="20">
         <v>411.647057562665</v>
       </c>
-      <c r="T37" s="23"/>
+      <c r="T37" s="19"/>
     </row>
     <row r="38" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O38" s="23">
+      <c r="O38" s="19">
         <v>20</v>
       </c>
-      <c r="P38" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q38" s="23">
-        <v>5</v>
-      </c>
-      <c r="R38" s="23">
+      <c r="P38" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q38" s="19">
+        <v>5</v>
+      </c>
+      <c r="R38" s="19">
         <v>3173.4</v>
       </c>
-      <c r="S38" s="24">
+      <c r="S38" s="20">
         <v>2075.80762596152</v>
       </c>
-      <c r="T38" s="23"/>
+      <c r="T38" s="19"/>
     </row>
     <row r="39" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O39" s="23">
+      <c r="O39" s="19">
         <v>20</v>
       </c>
-      <c r="P39" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q39" s="23">
-        <v>5</v>
-      </c>
-      <c r="R39" s="23">
+      <c r="P39" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q39" s="19">
+        <v>5</v>
+      </c>
+      <c r="R39" s="19">
         <v>5169.8</v>
       </c>
-      <c r="S39" s="24">
+      <c r="S39" s="20">
         <v>2464.669288160178</v>
       </c>
-      <c r="T39" s="23"/>
+      <c r="T39" s="19"/>
     </row>
     <row r="40" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O40" s="23">
+      <c r="O40" s="19">
         <v>20</v>
       </c>
-      <c r="P40" s="23">
-        <v>5</v>
-      </c>
-      <c r="Q40" s="23">
-        <v>5</v>
-      </c>
-      <c r="R40" s="23">
+      <c r="P40" s="19">
+        <v>5</v>
+      </c>
+      <c r="Q40" s="19">
+        <v>5</v>
+      </c>
+      <c r="R40" s="19">
         <v>7226</v>
       </c>
-      <c r="S40" s="24">
+      <c r="S40" s="20">
         <v>1863.650718348264</v>
       </c>
-      <c r="T40" s="23"/>
+      <c r="T40" s="19"/>
     </row>
     <row r="41" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O41" s="23"/>
-      <c r="P41" s="23"/>
-      <c r="Q41" s="23"/>
-      <c r="R41" s="23"/>
-      <c r="S41" s="23"/>
-      <c r="T41" s="23"/>
+      <c r="O41" s="19"/>
+      <c r="P41" s="19"/>
+      <c r="Q41" s="19"/>
+      <c r="R41" s="19"/>
+      <c r="S41" s="19"/>
+      <c r="T41" s="19"/>
     </row>
     <row r="42" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O42" s="22" t="s">
+      <c r="O42" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P42" s="22" t="s">
+      <c r="P42" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q42" s="22" t="s">
+      <c r="Q42" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R42" s="22" t="s">
+      <c r="R42" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S42" s="22" t="s">
+      <c r="S42" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T42" s="23"/>
+      <c r="T42" s="19"/>
     </row>
     <row r="43" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O43" s="23">
+      <c r="O43" s="19">
         <v>20</v>
       </c>
-      <c r="P43" s="23">
+      <c r="P43" s="19">
         <v>10</v>
       </c>
-      <c r="Q43" s="23">
-        <v>5</v>
-      </c>
-      <c r="R43" s="23">
+      <c r="Q43" s="19">
+        <v>5</v>
+      </c>
+      <c r="R43" s="19">
         <v>1250.4000000000001</v>
       </c>
-      <c r="S43" s="24">
+      <c r="S43" s="20">
         <v>416.45804110378282</v>
       </c>
-      <c r="T43" s="23"/>
+      <c r="T43" s="19"/>
     </row>
     <row r="44" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O44" s="23">
+      <c r="O44" s="19">
         <v>20</v>
       </c>
-      <c r="P44" s="23">
+      <c r="P44" s="19">
         <v>10</v>
       </c>
-      <c r="Q44" s="23">
-        <v>5</v>
-      </c>
-      <c r="R44" s="23">
+      <c r="Q44" s="19">
+        <v>5</v>
+      </c>
+      <c r="R44" s="19">
         <v>2595</v>
       </c>
-      <c r="S44" s="24">
+      <c r="S44" s="20">
         <v>1007.119655254528</v>
       </c>
-      <c r="T44" s="23"/>
+      <c r="T44" s="19"/>
     </row>
     <row r="45" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O45" s="23">
+      <c r="O45" s="19">
         <v>20</v>
       </c>
-      <c r="P45" s="23">
+      <c r="P45" s="19">
         <v>10</v>
       </c>
-      <c r="Q45" s="23">
-        <v>5</v>
-      </c>
-      <c r="R45" s="23">
+      <c r="Q45" s="19">
+        <v>5</v>
+      </c>
+      <c r="R45" s="19">
         <v>5128.2</v>
       </c>
-      <c r="S45" s="24">
+      <c r="S45" s="20">
         <v>1730.474559188895</v>
       </c>
-      <c r="T45" s="23"/>
+      <c r="T45" s="19"/>
     </row>
     <row r="46" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O46" s="23">
+      <c r="O46" s="19">
         <v>20</v>
       </c>
-      <c r="P46" s="23">
+      <c r="P46" s="19">
         <v>10</v>
       </c>
-      <c r="Q46" s="23">
-        <v>5</v>
-      </c>
-      <c r="R46" s="23">
+      <c r="Q46" s="19">
+        <v>5</v>
+      </c>
+      <c r="R46" s="19">
         <v>7963</v>
       </c>
-      <c r="S46" s="24">
+      <c r="S46" s="20">
         <v>360.91203914527432</v>
       </c>
-      <c r="T46" s="23"/>
+      <c r="T46" s="19"/>
     </row>
     <row r="47" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O47" s="23"/>
-      <c r="P47" s="23"/>
-      <c r="Q47" s="23"/>
-      <c r="R47" s="23"/>
-      <c r="S47" s="23"/>
-      <c r="T47" s="23"/>
+      <c r="O47" s="19"/>
+      <c r="P47" s="19"/>
+      <c r="Q47" s="19"/>
+      <c r="R47" s="19"/>
+      <c r="S47" s="19"/>
+      <c r="T47" s="19"/>
     </row>
     <row r="48" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O48" s="22" t="s">
+      <c r="O48" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P48" s="22" t="s">
+      <c r="P48" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q48" s="22" t="s">
+      <c r="Q48" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R48" s="22" t="s">
+      <c r="R48" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S48" s="22" t="s">
+      <c r="S48" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T48" s="23"/>
+      <c r="T48" s="19"/>
     </row>
     <row r="49" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O49" s="23">
+      <c r="O49" s="19">
         <v>20</v>
       </c>
-      <c r="P49" s="23">
+      <c r="P49" s="19">
         <v>15</v>
       </c>
-      <c r="Q49" s="23">
-        <v>5</v>
-      </c>
-      <c r="R49" s="23">
+      <c r="Q49" s="19">
+        <v>5</v>
+      </c>
+      <c r="R49" s="19">
         <v>788</v>
       </c>
-      <c r="S49" s="24">
+      <c r="S49" s="20">
         <v>314.48449882307398</v>
       </c>
-      <c r="T49" s="23"/>
+      <c r="T49" s="19"/>
     </row>
     <row r="50" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O50" s="23">
+      <c r="O50" s="19">
         <v>20</v>
       </c>
-      <c r="P50" s="23">
+      <c r="P50" s="19">
         <v>15</v>
       </c>
-      <c r="Q50" s="23">
-        <v>5</v>
-      </c>
-      <c r="R50" s="23">
+      <c r="Q50" s="19">
+        <v>5</v>
+      </c>
+      <c r="R50" s="19">
         <v>2736.8</v>
       </c>
-      <c r="S50" s="24">
+      <c r="S50" s="20">
         <v>867.92551523733891</v>
       </c>
-      <c r="T50" s="23"/>
+      <c r="T50" s="19"/>
     </row>
     <row r="51" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O51" s="23">
+      <c r="O51" s="19">
         <v>20</v>
       </c>
-      <c r="P51" s="23">
+      <c r="P51" s="19">
         <v>15</v>
       </c>
-      <c r="Q51" s="23">
-        <v>5</v>
-      </c>
-      <c r="R51" s="23">
+      <c r="Q51" s="19">
+        <v>5</v>
+      </c>
+      <c r="R51" s="19">
         <v>7839.4</v>
       </c>
-      <c r="S51" s="24">
+      <c r="S51" s="20">
         <v>5580.0229659025599</v>
       </c>
-      <c r="T51" s="23"/>
+      <c r="T51" s="19"/>
     </row>
     <row r="52" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O52" s="23">
+      <c r="O52" s="19">
         <v>20</v>
       </c>
-      <c r="P52" s="23">
+      <c r="P52" s="19">
         <v>15</v>
       </c>
-      <c r="Q52" s="23">
-        <v>5</v>
-      </c>
-      <c r="R52" s="23">
+      <c r="Q52" s="19">
+        <v>5</v>
+      </c>
+      <c r="R52" s="19">
         <v>9183.4</v>
       </c>
-      <c r="S52" s="24">
+      <c r="S52" s="20">
         <v>3811.277909048355</v>
       </c>
-      <c r="T52" s="23"/>
+      <c r="T52" s="19"/>
     </row>
     <row r="53" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O53" s="23"/>
-      <c r="P53" s="23"/>
-      <c r="Q53" s="23"/>
-      <c r="R53" s="23"/>
-      <c r="S53" s="23"/>
-      <c r="T53" s="23"/>
+      <c r="O53" s="19"/>
+      <c r="P53" s="19"/>
+      <c r="Q53" s="19"/>
+      <c r="R53" s="19"/>
+      <c r="S53" s="19"/>
+      <c r="T53" s="19"/>
     </row>
     <row r="54" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O54" s="22" t="s">
+      <c r="O54" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P54" s="22" t="s">
+      <c r="P54" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="Q54" s="22" t="s">
+      <c r="Q54" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="R54" s="22" t="s">
+      <c r="R54" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S54" s="22" t="s">
+      <c r="S54" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="T54" s="23"/>
+      <c r="T54" s="19"/>
     </row>
     <row r="55" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O55" s="23">
+      <c r="O55" s="19">
         <v>20</v>
       </c>
-      <c r="P55" s="23">
+      <c r="P55" s="19">
         <v>20</v>
       </c>
-      <c r="Q55" s="23">
-        <v>5</v>
-      </c>
-      <c r="R55" s="23">
+      <c r="Q55" s="19">
+        <v>5</v>
+      </c>
+      <c r="R55" s="19">
         <v>1139</v>
       </c>
-      <c r="S55" s="24">
+      <c r="S55" s="20">
         <v>409.11612043526219</v>
       </c>
-      <c r="T55" s="23"/>
+      <c r="T55" s="19"/>
     </row>
     <row r="56" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O56" s="23">
+      <c r="O56" s="19">
         <v>20</v>
       </c>
-      <c r="P56" s="23">
+      <c r="P56" s="19">
         <v>20</v>
       </c>
-      <c r="Q56" s="23">
-        <v>5</v>
-      </c>
-      <c r="R56" s="23">
+      <c r="Q56" s="19">
+        <v>5</v>
+      </c>
+      <c r="R56" s="19">
         <v>2293.4</v>
       </c>
-      <c r="S56" s="24">
+      <c r="S56" s="20">
         <v>944.16063251970002</v>
       </c>
-      <c r="T56" s="23"/>
+      <c r="T56" s="19"/>
     </row>
     <row r="57" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O57" s="23">
+      <c r="O57" s="19">
         <v>20</v>
       </c>
-      <c r="P57" s="23">
+      <c r="P57" s="19">
         <v>20</v>
       </c>
-      <c r="Q57" s="23">
-        <v>5</v>
-      </c>
-      <c r="R57" s="23">
+      <c r="Q57" s="19">
+        <v>5</v>
+      </c>
+      <c r="R57" s="19">
         <v>6469.4</v>
       </c>
-      <c r="S57" s="24">
+      <c r="S57" s="20">
         <v>2918.0354350144548</v>
       </c>
-      <c r="T57" s="23"/>
+      <c r="T57" s="19"/>
     </row>
     <row r="58" spans="15:20" x14ac:dyDescent="0.55000000000000004">
-      <c r="O58" s="23">
+      <c r="O58" s="19">
         <v>20</v>
       </c>
-      <c r="P58" s="23">
+      <c r="P58" s="19">
         <v>20</v>
       </c>
-      <c r="Q58" s="23">
-        <v>5</v>
-      </c>
-      <c r="R58" s="23">
+      <c r="Q58" s="19">
+        <v>5</v>
+      </c>
+      <c r="R58" s="19">
         <v>8850</v>
       </c>
-      <c r="S58" s="24">
+      <c r="S58" s="20">
         <v>1524.9044232344529</v>
       </c>
-      <c r="T58" s="23"/>
+      <c r="T58" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>